<commit_message>
Excel'lerden erisim sayfasi ve sutunu kaldirildi, jenerik trafik tanimi netlestirildi
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/cikti/appletv-rakip-trafigi.xlsx
+++ b/cikti/appletv-rakip-trafigi.xlsx
@@ -75563,12 +75563,12 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>Jenerik sayfa</t>
+          <t>Jenerik Sayfa Trafiği</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Dizinin kendi sayfası olmayan sonuç: platformların genel katalog sayfaları (tvplus.com.tr/dizi-izle gibi) ve aynı adı taşıyan başka yapımlar. Trafikleri dizi toplamına yazılmaz, 'Tüm SERP Sonuçları' sayfasında Kapsam sütununda işaretlidir.</t>
+          <t>Aramanın ilk 10'una giren ama dizinin kendi sayfası OLMAYAN sonuçların trafiği. İki kaynağı var: (1) platformların genel katalog sayfaları — 'now and then izle' sorgusunda nowtv.com.tr/film-izle 10. sırada çıkıyor ve kendi 8.266 trafiğini getiriyor; (2) aynı adı taşıyan başka yapımlar — aynı sorguda Now &amp; Later (2011) filminin sayfası. Bu trafik dizinin izleme talebine yazılamaz, o yüzden İzleme Odaklı Trafik'e girmez; kaç trafiğin bu şekilde elendiğini görebilmek için ayrı sütunda tutulur. Satır bazında 'Tüm SERP Sonuçları' sayfasında Kapsam sütununda işaretlidir.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Excel: Jenerik Sayfa Trafigi sutunu kaldirildi
Kural toplamlari hala belirledigi icin Yontem sayfasinda "Kapsam disi
sonuclar" notu kaldi; satir bazinda isaret Tum SERP Sonuclari sayfasindaki
Kapsam sutununda duruyor.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/cikti/appletv-rakip-trafigi.xlsx
+++ b/cikti/appletv-rakip-trafigi.xlsx
@@ -14,7 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Yöntem" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Dizi Bazında Trafik'!$A$1:$L$151</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Dizi Bazında Trafik'!$A$1:$K$151</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tüm SERP Sonuçları'!$A$1:$J$1421</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Domain Özeti'!$A$1:$F$106</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Sınıf Özeti'!$A$1:$C$4</definedName>
@@ -464,7 +464,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L151"/>
+  <dimension ref="A1:K151"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -477,8 +477,7 @@
     <col width="16" customWidth="1" min="8" max="8"/>
     <col width="11" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="23" customWidth="1" min="11" max="11"/>
-    <col width="15" customWidth="1" min="12" max="12"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -534,11 +533,6 @@
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>Jenerik Sayfa Trafiği</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
           <t>Taranan Sayfa</t>
         </is>
       </c>
@@ -583,9 +577,6 @@
         <v>15098</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L2" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -629,9 +620,6 @@
         <v>7330</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L3" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -675,9 +663,6 @@
         <v>2137</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L4" s="3" t="n">
         <v>9</v>
       </c>
     </row>
@@ -721,9 +706,6 @@
         <v>6508</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L5" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -767,9 +749,6 @@
         <v>6630</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L6" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -813,9 +792,6 @@
         <v>6908</v>
       </c>
       <c r="K7" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L7" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -859,9 +835,6 @@
         <v>0</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>8634</v>
-      </c>
-      <c r="L8" s="3" t="n">
         <v>9</v>
       </c>
     </row>
@@ -905,9 +878,6 @@
         <v>3341</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L9" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -951,9 +921,6 @@
         <v>1309</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L10" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -997,9 +964,6 @@
         <v>2773</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L11" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -1043,9 +1007,6 @@
         <v>1462</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>275</v>
-      </c>
-      <c r="L12" s="3" t="n">
         <v>8</v>
       </c>
     </row>
@@ -1089,9 +1050,6 @@
         <v>1230</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L13" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -1135,9 +1093,6 @@
         <v>663</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L14" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -1181,9 +1136,6 @@
         <v>221</v>
       </c>
       <c r="K15" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L15" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -1227,9 +1179,6 @@
         <v>823</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>14</v>
-      </c>
-      <c r="L16" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -1273,9 +1222,6 @@
         <v>1272</v>
       </c>
       <c r="K17" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L17" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -1319,9 +1265,6 @@
         <v>1235</v>
       </c>
       <c r="K18" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L18" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -1365,9 +1308,6 @@
         <v>624</v>
       </c>
       <c r="K19" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L19" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -1411,9 +1351,6 @@
         <v>584</v>
       </c>
       <c r="K20" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L20" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -1457,9 +1394,6 @@
         <v>691</v>
       </c>
       <c r="K21" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L21" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -1503,9 +1437,6 @@
         <v>1</v>
       </c>
       <c r="K22" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L22" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -1549,9 +1480,6 @@
         <v>0</v>
       </c>
       <c r="K23" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L23" s="3" t="n">
         <v>8</v>
       </c>
     </row>
@@ -1595,9 +1523,6 @@
         <v>326</v>
       </c>
       <c r="K24" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L24" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -1641,9 +1566,6 @@
         <v>316</v>
       </c>
       <c r="K25" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L25" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -1687,9 +1609,6 @@
         <v>35</v>
       </c>
       <c r="K26" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L26" s="3" t="n">
         <v>8</v>
       </c>
     </row>
@@ -1733,9 +1652,6 @@
         <v>34</v>
       </c>
       <c r="K27" s="3" t="n">
-        <v>10587</v>
-      </c>
-      <c r="L27" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -1779,9 +1695,6 @@
         <v>226</v>
       </c>
       <c r="K28" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L28" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -1825,9 +1738,6 @@
         <v>207</v>
       </c>
       <c r="K29" s="3" t="n">
-        <v>275</v>
-      </c>
-      <c r="L29" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -1871,9 +1781,6 @@
         <v>149</v>
       </c>
       <c r="K30" s="3" t="n">
-        <v>226</v>
-      </c>
-      <c r="L30" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -1917,9 +1824,6 @@
         <v>47</v>
       </c>
       <c r="K31" s="3" t="n">
-        <v>51</v>
-      </c>
-      <c r="L31" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -1963,9 +1867,6 @@
         <v>171</v>
       </c>
       <c r="K32" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L32" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -2009,9 +1910,6 @@
         <v>0</v>
       </c>
       <c r="K33" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L33" s="3" t="n">
         <v>9</v>
       </c>
     </row>
@@ -2055,9 +1953,6 @@
         <v>0</v>
       </c>
       <c r="K34" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L34" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -2101,9 +1996,6 @@
         <v>64</v>
       </c>
       <c r="K35" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L35" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -2147,9 +2039,6 @@
         <v>150</v>
       </c>
       <c r="K36" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L36" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -2193,9 +2082,6 @@
         <v>0</v>
       </c>
       <c r="K37" s="3" t="n">
-        <v>28</v>
-      </c>
-      <c r="L37" s="3" t="n">
         <v>9</v>
       </c>
     </row>
@@ -2239,9 +2125,6 @@
         <v>141</v>
       </c>
       <c r="K38" s="3" t="n">
-        <v>3634</v>
-      </c>
-      <c r="L38" s="3" t="n">
         <v>9</v>
       </c>
     </row>
@@ -2285,9 +2168,6 @@
         <v>0</v>
       </c>
       <c r="K39" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L39" s="3" t="n">
         <v>8</v>
       </c>
     </row>
@@ -2331,9 +2211,6 @@
         <v>139</v>
       </c>
       <c r="K40" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L40" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -2377,9 +2254,6 @@
         <v>111</v>
       </c>
       <c r="K41" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L41" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -2423,9 +2297,6 @@
         <v>80</v>
       </c>
       <c r="K42" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L42" s="3" t="n">
         <v>7</v>
       </c>
     </row>
@@ -2469,9 +2340,6 @@
         <v>0</v>
       </c>
       <c r="K43" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L43" s="3" t="n">
         <v>9</v>
       </c>
     </row>
@@ -2515,9 +2383,6 @@
         <v>1</v>
       </c>
       <c r="K44" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L44" s="3" t="n">
         <v>9</v>
       </c>
     </row>
@@ -2561,9 +2426,6 @@
         <v>70</v>
       </c>
       <c r="K45" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L45" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -2607,9 +2469,6 @@
         <v>0</v>
       </c>
       <c r="K46" s="3" t="n">
-        <v>197957</v>
-      </c>
-      <c r="L46" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -2653,9 +2512,6 @@
         <v>11</v>
       </c>
       <c r="K47" s="3" t="n">
-        <v>14</v>
-      </c>
-      <c r="L47" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -2699,9 +2555,6 @@
         <v>7</v>
       </c>
       <c r="K48" s="3" t="n">
-        <v>172</v>
-      </c>
-      <c r="L48" s="3" t="n">
         <v>8</v>
       </c>
     </row>
@@ -2745,9 +2598,6 @@
         <v>57</v>
       </c>
       <c r="K49" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L49" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -2791,9 +2641,6 @@
         <v>0</v>
       </c>
       <c r="K50" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L50" s="3" t="n">
         <v>9</v>
       </c>
     </row>
@@ -2837,9 +2684,6 @@
         <v>51</v>
       </c>
       <c r="K51" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L51" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -2883,9 +2727,6 @@
         <v>46</v>
       </c>
       <c r="K52" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L52" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -2929,9 +2770,6 @@
         <v>49</v>
       </c>
       <c r="K53" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L53" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -2975,9 +2813,6 @@
         <v>39</v>
       </c>
       <c r="K54" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L54" s="3" t="n">
         <v>9</v>
       </c>
     </row>
@@ -3021,9 +2856,6 @@
         <v>29</v>
       </c>
       <c r="K55" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L55" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -3067,9 +2899,6 @@
         <v>1</v>
       </c>
       <c r="K56" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L56" s="3" t="n">
         <v>8</v>
       </c>
     </row>
@@ -3113,9 +2942,6 @@
         <v>0</v>
       </c>
       <c r="K57" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L57" s="3" t="n">
         <v>9</v>
       </c>
     </row>
@@ -3159,9 +2985,6 @@
         <v>24</v>
       </c>
       <c r="K58" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L58" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -3205,9 +3028,6 @@
         <v>31</v>
       </c>
       <c r="K59" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L59" s="3" t="n">
         <v>8</v>
       </c>
     </row>
@@ -3251,9 +3071,6 @@
         <v>29</v>
       </c>
       <c r="K60" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L60" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -3297,9 +3114,6 @@
         <v>22</v>
       </c>
       <c r="K61" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L61" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -3343,9 +3157,6 @@
         <v>12</v>
       </c>
       <c r="K62" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L62" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -3389,9 +3200,6 @@
         <v>0</v>
       </c>
       <c r="K63" s="3" t="n">
-        <v>35638</v>
-      </c>
-      <c r="L63" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -3435,9 +3243,6 @@
         <v>0</v>
       </c>
       <c r="K64" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L64" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -3481,9 +3286,6 @@
         <v>10</v>
       </c>
       <c r="K65" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L65" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -3527,9 +3329,6 @@
         <v>20</v>
       </c>
       <c r="K66" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L66" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -3573,9 +3372,6 @@
         <v>7</v>
       </c>
       <c r="K67" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L67" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -3619,9 +3415,6 @@
         <v>0</v>
       </c>
       <c r="K68" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L68" s="3" t="n">
         <v>8</v>
       </c>
     </row>
@@ -3665,9 +3458,6 @@
         <v>0</v>
       </c>
       <c r="K69" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L69" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -3711,9 +3501,6 @@
         <v>9</v>
       </c>
       <c r="K70" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L70" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -3757,9 +3544,6 @@
         <v>8</v>
       </c>
       <c r="K71" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L71" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -3803,9 +3587,6 @@
         <v>0</v>
       </c>
       <c r="K72" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L72" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -3849,9 +3630,6 @@
         <v>6</v>
       </c>
       <c r="K73" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L73" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -3895,9 +3673,6 @@
         <v>0</v>
       </c>
       <c r="K74" s="3" t="n">
-        <v>8</v>
-      </c>
-      <c r="L74" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -3941,9 +3716,6 @@
         <v>10</v>
       </c>
       <c r="K75" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L75" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -3987,9 +3759,6 @@
         <v>8</v>
       </c>
       <c r="K76" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L76" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -4033,9 +3802,6 @@
         <v>1</v>
       </c>
       <c r="K77" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L77" s="3" t="n">
         <v>9</v>
       </c>
     </row>
@@ -4079,9 +3845,6 @@
         <v>0</v>
       </c>
       <c r="K78" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L78" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -4125,9 +3888,6 @@
         <v>8</v>
       </c>
       <c r="K79" s="3" t="n">
-        <v>9</v>
-      </c>
-      <c r="L79" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -4171,9 +3931,6 @@
         <v>9</v>
       </c>
       <c r="K80" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L80" s="3" t="n">
         <v>7</v>
       </c>
     </row>
@@ -4217,9 +3974,6 @@
         <v>0</v>
       </c>
       <c r="K81" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L81" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -4263,9 +4017,6 @@
         <v>5</v>
       </c>
       <c r="K82" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L82" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -4309,9 +4060,6 @@
         <v>7</v>
       </c>
       <c r="K83" s="3" t="n">
-        <v>40</v>
-      </c>
-      <c r="L83" s="3" t="n">
         <v>9</v>
       </c>
     </row>
@@ -4355,9 +4103,6 @@
         <v>6</v>
       </c>
       <c r="K84" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L84" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -4401,9 +4146,6 @@
         <v>1</v>
       </c>
       <c r="K85" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L85" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -4447,9 +4189,6 @@
         <v>2</v>
       </c>
       <c r="K86" s="3" t="n">
-        <v>477</v>
-      </c>
-      <c r="L86" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -4493,9 +4232,6 @@
         <v>4</v>
       </c>
       <c r="K87" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L87" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -4539,9 +4275,6 @@
         <v>0</v>
       </c>
       <c r="K88" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L88" s="3" t="n">
         <v>7</v>
       </c>
     </row>
@@ -4585,9 +4318,6 @@
         <v>4</v>
       </c>
       <c r="K89" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L89" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -4631,9 +4361,6 @@
         <v>0</v>
       </c>
       <c r="K90" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L90" s="3" t="n">
         <v>8</v>
       </c>
     </row>
@@ -4677,9 +4404,6 @@
         <v>2</v>
       </c>
       <c r="K91" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L91" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -4723,9 +4447,6 @@
         <v>2</v>
       </c>
       <c r="K92" s="3" t="n">
-        <v>8647</v>
-      </c>
-      <c r="L92" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -4769,9 +4490,6 @@
         <v>0</v>
       </c>
       <c r="K93" s="3" t="n">
-        <v>35638</v>
-      </c>
-      <c r="L93" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -4815,9 +4533,6 @@
         <v>2</v>
       </c>
       <c r="K94" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L94" s="3" t="n">
         <v>9</v>
       </c>
     </row>
@@ -4861,9 +4576,6 @@
         <v>0</v>
       </c>
       <c r="K95" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L95" s="3" t="n">
         <v>9</v>
       </c>
     </row>
@@ -4907,9 +4619,6 @@
         <v>0</v>
       </c>
       <c r="K96" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L96" s="3" t="n">
         <v>8</v>
       </c>
     </row>
@@ -4953,9 +4662,6 @@
         <v>0</v>
       </c>
       <c r="K97" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L97" s="3" t="n">
         <v>7</v>
       </c>
     </row>
@@ -4999,9 +4705,6 @@
         <v>1</v>
       </c>
       <c r="K98" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L98" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -5045,9 +4748,6 @@
         <v>1</v>
       </c>
       <c r="K99" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L99" s="3" t="n">
         <v>9</v>
       </c>
     </row>
@@ -5091,9 +4791,6 @@
         <v>0</v>
       </c>
       <c r="K100" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L100" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -5137,9 +4834,6 @@
         <v>0</v>
       </c>
       <c r="K101" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L101" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -5183,9 +4877,6 @@
         <v>0</v>
       </c>
       <c r="K102" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L102" s="3" t="n">
         <v>9</v>
       </c>
     </row>
@@ -5229,9 +4920,6 @@
         <v>1</v>
       </c>
       <c r="K103" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L103" s="3" t="n">
         <v>8</v>
       </c>
     </row>
@@ -5275,9 +4963,6 @@
         <v>1</v>
       </c>
       <c r="K104" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L104" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -5321,9 +5006,6 @@
         <v>0</v>
       </c>
       <c r="K105" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L105" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -5367,9 +5049,6 @@
         <v>1</v>
       </c>
       <c r="K106" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L106" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -5413,9 +5092,6 @@
         <v>1</v>
       </c>
       <c r="K107" s="3" t="n">
-        <v>195396</v>
-      </c>
-      <c r="L107" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -5459,9 +5135,6 @@
         <v>0</v>
       </c>
       <c r="K108" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L108" s="3" t="n">
         <v>9</v>
       </c>
     </row>
@@ -5505,9 +5178,6 @@
         <v>1</v>
       </c>
       <c r="K109" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L109" s="3" t="n">
         <v>9</v>
       </c>
     </row>
@@ -5551,9 +5221,6 @@
         <v>0</v>
       </c>
       <c r="K110" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L110" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -5597,9 +5264,6 @@
         <v>0</v>
       </c>
       <c r="K111" s="3" t="n">
-        <v>66</v>
-      </c>
-      <c r="L111" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -5643,9 +5307,6 @@
         <v>0</v>
       </c>
       <c r="K112" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L112" s="3" t="n">
         <v>9</v>
       </c>
     </row>
@@ -5689,9 +5350,6 @@
         <v>0</v>
       </c>
       <c r="K113" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L113" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -5735,9 +5393,6 @@
         <v>0</v>
       </c>
       <c r="K114" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L114" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -5781,9 +5436,6 @@
         <v>0</v>
       </c>
       <c r="K115" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L115" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -5827,9 +5479,6 @@
         <v>0</v>
       </c>
       <c r="K116" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L116" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -5873,9 +5522,6 @@
         <v>0</v>
       </c>
       <c r="K117" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L117" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -5919,9 +5565,6 @@
         <v>0</v>
       </c>
       <c r="K118" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L118" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -5965,9 +5608,6 @@
         <v>0</v>
       </c>
       <c r="K119" s="3" t="n">
-        <v>5850</v>
-      </c>
-      <c r="L119" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -6011,9 +5651,6 @@
         <v>0</v>
       </c>
       <c r="K120" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="L120" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -6057,9 +5694,6 @@
         <v>0</v>
       </c>
       <c r="K121" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L121" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -6103,9 +5737,6 @@
         <v>0</v>
       </c>
       <c r="K122" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L122" s="3" t="n">
         <v>8</v>
       </c>
     </row>
@@ -6149,9 +5780,6 @@
         <v>0</v>
       </c>
       <c r="K123" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L123" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -6195,9 +5823,6 @@
         <v>0</v>
       </c>
       <c r="K124" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L124" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -6241,9 +5866,6 @@
         <v>0</v>
       </c>
       <c r="K125" s="3" t="n">
-        <v>2137</v>
-      </c>
-      <c r="L125" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -6287,9 +5909,6 @@
         <v>0</v>
       </c>
       <c r="K126" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L126" s="3" t="n">
         <v>7</v>
       </c>
     </row>
@@ -6333,9 +5952,6 @@
         <v>0</v>
       </c>
       <c r="K127" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L127" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -6379,9 +5995,6 @@
         <v>0</v>
       </c>
       <c r="K128" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L128" s="3" t="n">
         <v>8</v>
       </c>
     </row>
@@ -6425,9 +6038,6 @@
         <v>0</v>
       </c>
       <c r="K129" s="3" t="n">
-        <v>75</v>
-      </c>
-      <c r="L129" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -6471,9 +6081,6 @@
         <v>0</v>
       </c>
       <c r="K130" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L130" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -6517,9 +6124,6 @@
         <v>0</v>
       </c>
       <c r="K131" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L131" s="3" t="n">
         <v>9</v>
       </c>
     </row>
@@ -6563,9 +6167,6 @@
         <v>0</v>
       </c>
       <c r="K132" s="3" t="n">
-        <v>80</v>
-      </c>
-      <c r="L132" s="3" t="n">
         <v>9</v>
       </c>
     </row>
@@ -6609,9 +6210,6 @@
         <v>0</v>
       </c>
       <c r="K133" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L133" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -6655,9 +6253,6 @@
         <v>0</v>
       </c>
       <c r="K134" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L134" s="3" t="n">
         <v>9</v>
       </c>
     </row>
@@ -6701,9 +6296,6 @@
         <v>0</v>
       </c>
       <c r="K135" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L135" s="3" t="n">
         <v>8</v>
       </c>
     </row>
@@ -6747,9 +6339,6 @@
         <v>0</v>
       </c>
       <c r="K136" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L136" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -6793,9 +6382,6 @@
         <v>0</v>
       </c>
       <c r="K137" s="3" t="n">
-        <v>1096</v>
-      </c>
-      <c r="L137" s="3" t="n">
         <v>9</v>
       </c>
     </row>
@@ -6839,9 +6425,6 @@
         <v>0</v>
       </c>
       <c r="K138" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L138" s="3" t="n">
         <v>9</v>
       </c>
     </row>
@@ -6885,9 +6468,6 @@
         <v>0</v>
       </c>
       <c r="K139" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="L139" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -6931,9 +6511,6 @@
         <v>0</v>
       </c>
       <c r="K140" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L140" s="3" t="n">
         <v>9</v>
       </c>
     </row>
@@ -6977,9 +6554,6 @@
         <v>0</v>
       </c>
       <c r="K141" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L141" s="3" t="n">
         <v>9</v>
       </c>
     </row>
@@ -7023,9 +6597,6 @@
         <v>0</v>
       </c>
       <c r="K142" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="L142" s="3" t="n">
         <v>9</v>
       </c>
     </row>
@@ -7069,9 +6640,6 @@
         <v>0</v>
       </c>
       <c r="K143" s="3" t="n">
-        <v>240349</v>
-      </c>
-      <c r="L143" s="3" t="n">
         <v>9</v>
       </c>
     </row>
@@ -7115,9 +6683,6 @@
         <v>0</v>
       </c>
       <c r="K144" s="3" t="n">
-        <v>2843</v>
-      </c>
-      <c r="L144" s="3" t="n">
         <v>9</v>
       </c>
     </row>
@@ -7161,9 +6726,6 @@
         <v>23</v>
       </c>
       <c r="K145" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L145" s="3" t="n">
         <v>9</v>
       </c>
     </row>
@@ -7207,9 +6769,6 @@
         <v>0</v>
       </c>
       <c r="K146" s="3" t="n">
-        <v>6</v>
-      </c>
-      <c r="L146" s="3" t="n">
         <v>8</v>
       </c>
     </row>
@@ -7253,9 +6812,6 @@
         <v>0</v>
       </c>
       <c r="K147" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L147" s="3" t="n">
         <v>8</v>
       </c>
     </row>
@@ -7299,9 +6855,6 @@
         <v>0</v>
       </c>
       <c r="K148" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L148" s="3" t="n">
         <v>10</v>
       </c>
     </row>
@@ -7345,9 +6898,6 @@
         <v>0</v>
       </c>
       <c r="K149" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L149" s="3" t="n">
         <v>8</v>
       </c>
     </row>
@@ -7391,9 +6941,6 @@
         <v>0</v>
       </c>
       <c r="K150" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L150" s="3" t="n">
         <v>9</v>
       </c>
     </row>
@@ -7437,14 +6984,11 @@
         <v>0</v>
       </c>
       <c r="K151" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L151" s="3" t="n">
         <v>10</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L151"/>
+  <autoFilter ref="A1:K151"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -75563,12 +75107,12 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>Jenerik Sayfa Trafiği</t>
+          <t>Kapsam dışı sonuçlar</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Aramanın ilk 10'una giren ama dizinin kendi sayfası OLMAYAN sonuçların trafiği. İki kaynağı var: (1) platformların genel katalog sayfaları — 'now and then izle' sorgusunda nowtv.com.tr/film-izle 10. sırada çıkıyor ve kendi 8.266 trafiğini getiriyor; (2) aynı adı taşıyan başka yapımlar — aynı sorguda Now &amp; Later (2011) filminin sayfası. Bu trafik dizinin izleme talebine yazılamaz, o yüzden İzleme Odaklı Trafik'e girmez; kaç trafiğin bu şekilde elendiğini görebilmek için ayrı sütunda tutulur. Satır bazında 'Tüm SERP Sonuçları' sayfasında Kapsam sütununda işaretlidir.</t>
+          <t>Aramanın ilk 10'una dizinin kendi sayfası olmayan sonuçlar da giriyor: platformların genel katalog sayfaları (nowtv.com.tr/film-izle gibi, kendi bütün trafiğini getirir) ve aynı adı taşıyan başka yapımlar. Bu satırların trafiği dizi toplamlarına katılmaz; 'Tüm SERP Sonuçları' sayfasında Kapsam sütununda 'Jenerik / başka yapım' olarak işaretlidir.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Excel sütun adları toplam/ortalama ve dönem bilgisini taşısın
- excel_hacim.py: Aylık Hacim (Google Ads ort.), Son 12 Ay Toplam, Son 12 Ay Aylık Ort.,
  Önceki 12 Ay Toplam, YoY % (toplam karşılaştırması); küme sayfalarında Aylık Hacim Toplamı
- excel_rakip.py: sorgu ve trafik sütunları aylık olduğunu adında söylüyor
- excel_ortak.py: başlığında % geçen sütuna #,##0.0 (21.398,8 değeri 21.399 görünüyordu)
- Her iki Yöntem sayfasına metrik tanımları ve dönem pencereleri

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/cikti/appletv-rakip-trafigi.xlsx
+++ b/cikti/appletv-rakip-trafigi.xlsx
@@ -471,12 +471,12 @@
     <col width="43" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="11" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="37" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
+    <col width="21" customWidth="1" min="7" max="7"/>
+    <col width="29" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
     <col width="15" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
@@ -503,32 +503,32 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Sorgu Hacmi</t>
+          <t>Sorgu Aylık Hacmi (Google Ads ort.)</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>İzleme Odaklı Trafik</t>
+          <t>İzleme Odaklı Aylık Trafik</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Korsan</t>
+          <t>Korsan Aylık Trafik</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Meşru Platform</t>
+          <t>Meşru Platform Aylık Trafik</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Agregatör</t>
+          <t>Agregatör Aylık Trafik</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>İlk 3 Trafiği</t>
+          <t>İlk 3 Aylık Trafik</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
@@ -7004,13 +7004,13 @@
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
     <col width="33" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="31" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
     <col width="60" customWidth="1" min="6" max="6"/>
     <col width="45" customWidth="1" min="7" max="7"/>
     <col width="19" customWidth="1" min="8" max="8"/>
-    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="35" customWidth="1" min="9" max="9"/>
     <col width="23" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
@@ -7027,7 +7027,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Aylık Hacim</t>
+          <t>Aylık Hacim (Google Ads ort.)</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -7057,7 +7057,7 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Ahrefs Sayfa Trafiği</t>
+          <t>Aylık Sayfa Trafiği (Ahrefs tah.)</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
@@ -72406,7 +72406,7 @@
     <col width="11" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="35" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -72437,7 +72437,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Ahrefs Sayfa Trafiği</t>
+          <t>Aylık Sayfa Trafiği (Ahrefs tah.)</t>
         </is>
       </c>
     </row>
@@ -74978,7 +74978,7 @@
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="35" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -74994,7 +74994,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Ahrefs Sayfa Trafiği</t>
+          <t>Aylık Sayfa Trafiği (Ahrefs tah.)</t>
         </is>
       </c>
     </row>
@@ -75049,7 +75049,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -75071,70 +75071,82 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>Sıralama kaynağı</t>
+          <t>Sütun adlarındaki dönem</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>DataForSEO · Google Türkiye (location 2792, dil tr, masaüstü), ilk 10 organik sonuç.</t>
+          <t>Bu dosyadaki tüm hacim ve trafik sütunları AYLIK büyüklüktür; 12 aylık toplam içermez. 'Google Ads ort.' aracın kendi ortalama aylık arama hacmi değeridir, 'Ahrefs tah.' ise sayfanın tahmini aylık organik trafiğidir.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>Trafik kaynağı</t>
+          <t>Sıralama kaynağı</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>Ahrefs batch-analysis, mode=exact. Değer o URL'in tahmini aylık organik trafiğidir; yalnızca bu sorgudan geleni değil, sayfanın tamamını kapsar. Üst sınır okuması verir.</t>
+          <t>DataForSEO · Google Türkiye (location 2792, dil tr, masaüstü), ilk 10 organik sonuç.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>İzleme odaklı trafik</t>
+          <t>Trafik kaynağı</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>Korsan + meşru platform sayfalarının toplamı. Agregatör ve bilgi siteleri (JustWatch, IMDb, Wikipedia) izleme sayfası sunmadığı için ayrı sütundadır.</t>
+          <t>Ahrefs batch-analysis, mode=exact. Değer o URL'in tahmini aylık organik trafiğidir; yalnızca bu sorgudan geleni değil, sayfanın tamamını kapsar. Üst sınır okuması verir.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>Kapsam dışı sonuçlar</t>
+          <t>İzleme odaklı trafik</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Aramanın ilk 10'una dizinin kendi sayfası olmayan sonuçlar da giriyor: platformların genel katalog sayfaları (nowtv.com.tr/film-izle gibi, kendi bütün trafiğini getirir) ve aynı adı taşıyan başka yapımlar. Bu satırların trafiği dizi toplamlarına katılmaz; 'Tüm SERP Sonuçları' sayfasında Kapsam sütununda 'Jenerik / başka yapım' olarak işaretlidir.</t>
+          <t>Korsan + meşru platform sayfalarının toplamı. Agregatör ve bilgi siteleri (JustWatch, IMDb, Wikipedia) izleme sayfası sunmadığı için ayrı sütundadır.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Sınır</t>
+          <t>Kapsam dışı sonuçlar</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Ad belirsizliği taşıyan dizilerde sayfa düzeyinde sızıntı sürebilir; ör. 'now and then' sorgusunda 1995 tarihli aynı adlı filmin platform sayfası ilk 10'a giriyor.</t>
+          <t>Aramanın ilk 10'una dizinin kendi sayfası olmayan sonuçlar da giriyor: platformların genel katalog sayfaları (nowtv.com.tr/film-izle gibi, kendi bütün trafiğini getirir) ve aynı adı taşıyan başka yapımlar. Bu satırların trafiği dizi toplamlarına katılmaz; 'Tüm SERP Sonuçları' sayfasında Kapsam sütununda 'Jenerik / başka yapım' olarak işaretlidir.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
+          <t>Sınır</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Ad belirsizliği taşıyan dizilerde sayfa düzeyinde sızıntı sürebilir; ör. 'now and then' sorgusunda 1995 tarihli aynı adlı filmin platform sayfası ilk 10'a giriyor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
           <t>Kaynak</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>Kaynak: DataForSEO (sıralama) · Ahrefs (sayfa trafiği)</t>
         </is>

</xml_diff>